<commit_message>
Refactor: Modularización del sistema, portabilidad de assets y separación de reportes
</commit_message>
<xml_diff>
--- a/Tables/Asesorías académicas (respuestas).xlsx
+++ b/Tables/Asesorías académicas (respuestas).xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_CV_test\H_System\Tables\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB26D44-3652-40A4-A9EF-28D51C6BE2A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Respuestas de formulario 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Respuestas de formulario 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="44">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -148,20 +157,29 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -170,76 +188,39 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF5B3F86"/>
-          <bgColor rgb="FF5B3F86"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8F9FA"/>
-          <bgColor rgb="FFF8F9FA"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -256,44 +237,68 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8F9FA"/>
+          <bgColor rgb="FFF8F9FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF5B3F86"/>
+          <bgColor rgb="FF5B3F86"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Respuestas de formulario 1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Respuestas de formulario 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H13" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:H16">
   <tableColumns count="8">
-    <tableColumn name="Marca temporal" id="1"/>
-    <tableColumn name="Dirección de correo electrónico" id="2"/>
-    <tableColumn name="No. de control" id="3"/>
-    <tableColumn name="Nombre del alumno(a)" id="4"/>
-    <tableColumn name="Sexo" id="5"/>
-    <tableColumn name="Nombre del asesor(a)" id="6"/>
-    <tableColumn name="Materia" id="7"/>
-    <tableColumn name="Tipo de asesoría" id="8"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Marca temporal"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Dirección de correo electrónico"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="No. de control"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Nombre del alumno(a)"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Sexo"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Nombre del asesor(a)"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Materia"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Tipo de asesoría"/>
   </tableColumns>
-  <tableStyleInfo name="Respuestas de formulario 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Respuestas de formulario 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -483,26 +488,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.88"/>
-    <col customWidth="1" min="2" max="2" width="27.88"/>
-    <col customWidth="1" min="3" max="3" width="18.88"/>
-    <col customWidth="1" min="4" max="4" width="21.63"/>
-    <col customWidth="1" min="5" max="5" width="18.88"/>
-    <col customWidth="1" min="6" max="6" width="21.13"/>
-    <col customWidth="1" min="7" max="14" width="18.88"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="18.88671875" customWidth="1"/>
+    <col min="6" max="6" width="21.109375" customWidth="1"/>
+    <col min="7" max="14" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,15 +536,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>46212.95362015047</v>
+        <v>46212.953620150467</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="3">
-        <v>3.23030001E8</v>
+        <v>323030001</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>9</v>
@@ -554,7 +562,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>46224.538542291666</v>
       </c>
@@ -562,7 +570,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="3">
-        <v>3.23030001E8</v>
+        <v>323030001</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>9</v>
@@ -580,15 +588,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>46224.53895402778</v>
+        <v>46224.538954027783</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="3">
-        <v>3.2303004E8</v>
+        <v>323030040</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>17</v>
@@ -606,7 +614,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>46224.539405752315</v>
       </c>
@@ -614,7 +622,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>3.2300301E8</v>
+        <v>323003010</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>21</v>
@@ -632,7 +640,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>46224.539408854165</v>
       </c>
@@ -640,7 +648,7 @@
         <v>24</v>
       </c>
       <c r="C6" s="3">
-        <v>3.23000511E8</v>
+        <v>323000511</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>25</v>
@@ -658,192 +666,273 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="4">
-        <v>46225.48563767361</v>
+    <row r="7" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46225.485637673613</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="5">
-        <v>3230345.0</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="3">
+        <v>3230345</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="4">
+    <row r="8" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
         <v>46225.486526249995</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="5">
-        <v>3420365.0</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="3">
+        <v>3420365</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="4">
-        <v>46225.48716371528</v>
+    <row r="9" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>46225.487163715283</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="5">
-        <v>3230316.0</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="C9" s="3">
+        <v>3230316</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="4">
-        <v>46225.48811006945</v>
+    <row r="10" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>46225.488110069447</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="5">
-        <v>3230678.0</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="C10" s="3">
+        <v>3230678</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="5" t="s">
+      <c r="G10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="4">
+    <row r="11" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
         <v>46225.488881377314</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="5">
-        <v>3245671.0</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="C11" s="3">
+        <v>3245671</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H11" s="5" t="s">
+      <c r="G11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="4">
-        <v>46225.49120259259</v>
+    <row r="12" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>46225.491202592588</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="5">
-        <v>3520586.0</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="C12" s="3">
+        <v>3520586</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H12" s="5" t="s">
+      <c r="G12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="4">
+    <row r="13" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
         <v>46225.49206866898</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="5">
-        <v>1527440.0</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="C13" s="3">
+        <v>1527440</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" s="5" t="s">
+      <c r="G13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>46272.953622685185</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14">
+        <v>323030001</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>46272.953622685185</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>323030001</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>46272.953622685185</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
+        <v>323030001</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5"/>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>